<commit_message>
DAX intro final commmit with all updates
</commit_message>
<xml_diff>
--- a/Excel/8_Power_pivot/3_DAX_Intro.xlsx
+++ b/Excel/8_Power_pivot/3_DAX_Intro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\data-analytics-learning\Excel\8_Power_pivot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A11BEA-0E2A-4BE0-B519-AB52183B6DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08B0640B-D1F6-465A-B3F7-85B913F844E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="763" activeTab="2" xr2:uid="{6F716FE0-A4DF-418B-900B-3408E44BFC15}"/>
   </bookViews>
@@ -268,25 +268,7 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     </dxf>
@@ -1076,7 +1058,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7201CCAA-D2F1-447A-8DBC-EC5FD29147B5}" type="CELLRANGE">
+                    <a:fld id="{50B1287E-3559-4E02-908C-3F1D05DA33CB}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1110,7 +1092,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5ED2342B-F1AA-40D5-AA9A-5A40A6AB69AF}" type="CELLRANGE">
+                    <a:fld id="{068C7AB4-78B0-4B95-9235-534E7EA03CD4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1144,7 +1126,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DCCCA8CD-D940-4B40-9857-54320644204D}" type="CELLRANGE">
+                    <a:fld id="{7F1F7A49-E8CF-47A2-A00C-AF5CBF0EAF0F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1178,7 +1160,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CAD70DBE-FEFA-4EEF-883A-6572C2AFE656}" type="CELLRANGE">
+                    <a:fld id="{D6E6F02D-C88E-4EAE-8124-E0228E2BF963}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1212,7 +1194,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9BDDB490-50BE-4107-84A9-DC4C231AAB69}" type="CELLRANGE">
+                    <a:fld id="{C1A0747A-6C7E-4495-9911-6359740593B4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1267,7 +1249,7 @@
                         <a:cs typeface="+mn-cs"/>
                       </a:defRPr>
                     </a:pPr>
-                    <a:fld id="{0FCF9E07-1145-4337-A0DD-B0221186E342}" type="CELLRANGE">
+                    <a:fld id="{B0F057F4-9247-442E-8B5C-8B25BB634394}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr>
                         <a:defRPr/>
@@ -1343,7 +1325,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{66567676-77A3-43BA-AD45-11439936A5C4}" type="CELLRANGE">
+                    <a:fld id="{2C995462-3679-4FC6-BCC6-255904D09B02}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1382,7 +1364,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7CE2E15F-7FE1-49A5-8564-E1193E688AB9}" type="CELLRANGE">
+                    <a:fld id="{3297992F-6FBB-4626-858F-6CF0C3DBCEA6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1421,7 +1403,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D1A98433-23CA-471A-9100-9ADEF7F399A8}" type="CELLRANGE">
+                    <a:fld id="{0096DF68-B17F-4CD9-A340-8772CE80A6A5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1460,7 +1442,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{37E3E9BE-0312-4A11-A69B-B4752EA7F1E5}" type="CELLRANGE">
+                    <a:fld id="{CA8EA5C8-3547-4101-B6D4-8D6DB0254303}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3675,7 +3657,7 @@
     <dataField fld="1" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="6">
+    <format dxfId="0">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>

</xml_diff>